<commit_message>
Binary search tree testing done.
</commit_message>
<xml_diff>
--- a/results/excel/task1_benchmark.xlsx
+++ b/results/excel/task1_benchmark.xlsx
@@ -437,7 +437,7 @@
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,16 +500,16 @@
         <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>5.30400313436985e-05</v>
+        <v>5.252000410109759e-05</v>
       </c>
       <c r="F2" t="n">
-        <v>8.610065905729366e-06</v>
+        <v>9.101999215495516e-06</v>
       </c>
       <c r="G2" t="n">
-        <v>4.820001777261496e-05</v>
+        <v>4.720001015812159e-05</v>
       </c>
       <c r="H2" t="n">
-        <v>6.84000551700592e-05</v>
+        <v>6.859994027763605e-05</v>
       </c>
     </row>
     <row r="3">
@@ -530,16 +530,16 @@
         <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0004333999939262867</v>
+        <v>0.0004660000093281269</v>
       </c>
       <c r="F3" t="n">
-        <v>2.71080572362993e-05</v>
+        <v>3.191216421387701e-05</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0004097999772056937</v>
+        <v>0.0004363999469205737</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0004795000422745943</v>
+        <v>0.0005098000401630998</v>
       </c>
     </row>
     <row r="4">
@@ -560,16 +560,16 @@
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0001503199804574251</v>
+        <v>0.0001574200112372637</v>
       </c>
       <c r="F4" t="n">
-        <v>1.73602088571671e-05</v>
+        <v>3.645414206995339e-05</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0001400000182911754</v>
+        <v>0.00013930001296103</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0001810999820008874</v>
+        <v>0.0002225999487563968</v>
       </c>
     </row>
     <row r="5">
@@ -590,16 +590,16 @@
         <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>7.064000237733126e-05</v>
+        <v>7.209999021142721e-05</v>
       </c>
       <c r="F5" t="n">
-        <v>6.777780666692196e-06</v>
+        <v>7.992783831991251e-06</v>
       </c>
       <c r="G5" t="n">
-        <v>6.7099928855896e-05</v>
+        <v>6.590003613382578e-05</v>
       </c>
       <c r="H5" t="n">
-        <v>8.270004764199257e-05</v>
+        <v>8.509994950145483e-05</v>
       </c>
     </row>
     <row r="6">
@@ -620,16 +620,16 @@
         <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001099899993278086</v>
+        <v>0.0008121600374579429</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0006285080032786166</v>
+        <v>8.709280035167184e-05</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0007919000927358866</v>
+        <v>0.0007537000346928835</v>
       </c>
       <c r="H6" t="n">
-        <v>0.002223299932666123</v>
+        <v>0.0009652000153437257</v>
       </c>
     </row>
     <row r="7">
@@ -650,16 +650,16 @@
         <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>0.009754240023903548</v>
+        <v>0.009993699984624982</v>
       </c>
       <c r="F7" t="n">
-        <v>0.001144939016693745</v>
+        <v>0.001514868116305719</v>
       </c>
       <c r="G7" t="n">
-        <v>0.008414000039920211</v>
+        <v>0.008553100051358342</v>
       </c>
       <c r="H7" t="n">
-        <v>0.01136040000710636</v>
+        <v>0.01212440000381321</v>
       </c>
     </row>
     <row r="8">
@@ -680,16 +680,16 @@
         <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>0.002019019983708859</v>
+        <v>0.001913939975202084</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0001695591323186722</v>
+        <v>0.0002152080701470673</v>
       </c>
       <c r="G8" t="n">
-        <v>0.001818299992009997</v>
+        <v>0.001655100029893219</v>
       </c>
       <c r="H8" t="n">
-        <v>0.002272199955768883</v>
+        <v>0.002203499898314476</v>
       </c>
     </row>
     <row r="9">
@@ -710,16 +710,16 @@
         <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>0.001014059991575778</v>
+        <v>0.0009691599756479263</v>
       </c>
       <c r="F9" t="n">
-        <v>5.129712650091081e-05</v>
+        <v>4.828368721308359e-05</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0009820000268518925</v>
+        <v>0.0009065999183803797</v>
       </c>
       <c r="H9" t="n">
-        <v>0.001104900031350553</v>
+        <v>0.001035799970850348</v>
       </c>
     </row>
     <row r="10">
@@ -740,16 +740,16 @@
         <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01942338002845645</v>
+        <v>0.01868201999459416</v>
       </c>
       <c r="F10" t="n">
-        <v>0.01144829148827991</v>
+        <v>0.0104253913728039</v>
       </c>
       <c r="G10" t="n">
-        <v>0.01324110000859946</v>
+        <v>0.0134566999040544</v>
       </c>
       <c r="H10" t="n">
-        <v>0.03986600006464869</v>
+        <v>0.03731399995740503</v>
       </c>
     </row>
     <row r="11">
@@ -770,16 +770,16 @@
         <v>5</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1190922200214118</v>
+        <v>0.1190036199986935</v>
       </c>
       <c r="F11" t="n">
-        <v>0.008505266778448456</v>
+        <v>0.007271224171018582</v>
       </c>
       <c r="G11" t="n">
-        <v>0.111445700051263</v>
+        <v>0.1135992999188602</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1308015999384224</v>
+        <v>0.1314558000303805</v>
       </c>
     </row>
     <row r="12">
@@ -800,16 +800,16 @@
         <v>5</v>
       </c>
       <c r="E12" t="n">
-        <v>0.04158062003552913</v>
+        <v>0.03096968003083021</v>
       </c>
       <c r="F12" t="n">
-        <v>0.01915105717000805</v>
+        <v>0.01730341055809139</v>
       </c>
       <c r="G12" t="n">
-        <v>0.01866880001034588</v>
+        <v>0.01759750000201166</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05757630011066794</v>
+        <v>0.05230710003525019</v>
       </c>
     </row>
     <row r="13">
@@ -830,16 +830,16 @@
         <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>0.01231152000837028</v>
+        <v>0.01591058000922203</v>
       </c>
       <c r="F13" t="n">
-        <v>0.002588439804827763</v>
+        <v>0.01167473456395753</v>
       </c>
       <c r="G13" t="n">
-        <v>0.01007079996634275</v>
+        <v>0.009173800004646182</v>
       </c>
       <c r="H13" t="n">
-        <v>0.01621150004211813</v>
+        <v>0.03672650002408773</v>
       </c>
     </row>
   </sheetData>
@@ -926,16 +926,16 @@
         <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>4.256002139300108e-05</v>
+        <v>4.081998486071825e-05</v>
       </c>
       <c r="F2" t="n">
-        <v>3.511838839610925e-06</v>
+        <v>3.743945110697013e-06</v>
       </c>
       <c r="G2" t="n">
-        <v>4.050007555633783e-05</v>
+        <v>3.879994619637728e-05</v>
       </c>
       <c r="H2" t="n">
-        <v>4.880002234131098e-05</v>
+        <v>4.75000124424696e-05</v>
       </c>
     </row>
     <row r="3">
@@ -956,16 +956,16 @@
         <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>3.877999261021614e-05</v>
+        <v>3.708000294864178e-05</v>
       </c>
       <c r="F3" t="n">
-        <v>3.384087569431525e-06</v>
+        <v>3.340943837580955e-06</v>
       </c>
       <c r="G3" t="n">
-        <v>3.66999302059412e-05</v>
+        <v>3.510003443807364e-05</v>
       </c>
       <c r="H3" t="n">
-        <v>4.469999112188816e-05</v>
+        <v>4.299997817724943e-05</v>
       </c>
     </row>
     <row r="4">
@@ -986,16 +986,16 @@
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>2.043999265879393e-05</v>
+        <v>1.87800033017993e-05</v>
       </c>
       <c r="F4" t="n">
-        <v>2.642525723929926e-06</v>
+        <v>2.701329268085013e-06</v>
       </c>
       <c r="G4" t="n">
-        <v>1.859990879893303e-05</v>
+        <v>1.670001074671745e-05</v>
       </c>
       <c r="H4" t="n">
-        <v>2.509995829313993e-05</v>
+        <v>2.350006252527237e-05</v>
       </c>
     </row>
     <row r="5">
@@ -1016,16 +1016,16 @@
         <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0001205599866807461</v>
+        <v>0.0001195400021970272</v>
       </c>
       <c r="F5" t="n">
-        <v>4.619276326335012e-06</v>
+        <v>1.124602087025753e-05</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0001182999694719911</v>
+        <v>0.0001103000249713659</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0001287999330088496</v>
+        <v>0.0001377000007778406</v>
       </c>
     </row>
     <row r="6">
@@ -1046,16 +1046,16 @@
         <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0001199600053951144</v>
+        <v>0.0001133800018578768</v>
       </c>
       <c r="F6" t="n">
-        <v>4.763727894171659e-06</v>
+        <v>7.423419418831906e-06</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0001158000668510795</v>
+        <v>0.0001091000158339739</v>
       </c>
       <c r="H6" t="n">
-        <v>0.000126900034956634</v>
+        <v>0.0001265000319108367</v>
       </c>
     </row>
     <row r="7">
@@ -1076,16 +1076,16 @@
         <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>5.216000135987997e-05</v>
+        <v>5.123999435454607e-05</v>
       </c>
       <c r="F7" t="n">
-        <v>6.070676585176572e-06</v>
+        <v>2.424068014341225e-05</v>
       </c>
       <c r="G7" t="n">
-        <v>4.899990744888783e-05</v>
+        <v>4.0199956856668e-05</v>
       </c>
       <c r="H7" t="n">
-        <v>6.300001405179501e-05</v>
+        <v>9.459990542382002e-05</v>
       </c>
     </row>
     <row r="8">
@@ -1106,16 +1106,16 @@
         <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0001367200398817658</v>
+        <v>9.570000693202019e-05</v>
       </c>
       <c r="F8" t="n">
-        <v>3.375045547324298e-05</v>
+        <v>4.718034554045916e-06</v>
       </c>
       <c r="G8" t="n">
-        <v>9.96000599116087e-05</v>
+        <v>9.290000889450312e-05</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0001790000824257731</v>
+        <v>0.000104099977761507</v>
       </c>
     </row>
     <row r="9">
@@ -1136,16 +1136,16 @@
         <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0001974599668756127</v>
+        <v>0.000108579988591373</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0001069061413039811</v>
+        <v>1.049628811986195e-05</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0001080000074580312</v>
+        <v>0.0001011000713333488</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0003829998895525932</v>
+        <v>0.000125700025819242</v>
       </c>
     </row>
     <row r="10">
@@ -1166,16 +1166,16 @@
         <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>5.324000958353281e-05</v>
+        <v>5.085999146103859e-05</v>
       </c>
       <c r="F10" t="n">
-        <v>3.726736704707816e-05</v>
+        <v>3.177724817245472e-05</v>
       </c>
       <c r="G10" t="n">
-        <v>3.620004281401634e-05</v>
+        <v>3.599992487579584e-05</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0001199000980705023</v>
+        <v>0.0001077000051736832</v>
       </c>
     </row>
   </sheetData>

</xml_diff>